<commit_message>
ready core without interface
</commit_message>
<xml_diff>
--- a/user_table/test.xlsx
+++ b/user_table/test.xlsx
@@ -413,247 +413,273 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>WORK_ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>WORK_ID</t>
+          <t>E1 N1</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>E1 N1</t>
+          <t>E1 N2</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>E1 N2</t>
+          <t>E1 N3</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>E1 N3</t>
+          <t>E1 N4</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>E1 N4</t>
+          <t>E1 N5</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>E1 N5</t>
+          <t>E1 N6</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>E1 N6</t>
+          <t>E2 N1</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>E2 N1</t>
+          <t>E2 N2</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>E2 N2</t>
+          <t>E2 N3</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>E2 N3</t>
+          <t>E2 N4</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>E2 N4</t>
+          <t>E2 N5</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>E2 N5</t>
+          <t>E2 N6</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>E2 N6</t>
+          <t>id_exp1</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>id_exp1</t>
+          <t>id_exp2</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>id_exp2</t>
+          <t>mistake</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>n_w_mistake</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>111111111111</v>
       </c>
       <c r="B2" t="n">
-        <v>111111111111</v>
+        <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
       </c>
       <c r="L2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N2" t="n">
-        <v>2</v>
+        <v>1488902412421</v>
       </c>
       <c r="O2" t="n">
-        <v>1488902412421</v>
+        <v>133722813124940</v>
       </c>
       <c r="P2" t="n">
-        <v>133722813124940</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>22222222222</v>
       </c>
       <c r="B3" t="n">
-        <v>22222222222</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
         <v>3</v>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
         <v>3</v>
       </c>
-      <c r="F3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2</v>
-      </c>
       <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" t="n">
         <v>3</v>
       </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="n">
-        <v>4</v>
-      </c>
-      <c r="L3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M3" t="n">
-        <v>2</v>
-      </c>
       <c r="N3" t="n">
-        <v>3</v>
+        <v>1488902412421</v>
       </c>
       <c r="O3" t="n">
-        <v>1488902412421</v>
+        <v>133722813124940</v>
       </c>
       <c r="P3" t="n">
-        <v>133722813124940</v>
+        <v>2</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 2 </t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
+        <v>33333333333</v>
+      </c>
+      <c r="B4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
-        <v>33333333333</v>
-      </c>
       <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
         <v>3</v>
       </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
       <c r="L4" t="n">
-        <v>3</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
+        <v>0</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
       </c>
       <c r="N4" t="n">
-        <v>1</v>
+        <v>1488902412421</v>
       </c>
       <c r="O4" t="n">
-        <v>1488902412421</v>
+        <v>133722813124940</v>
       </c>
       <c r="P4" t="n">
-        <v>133722813124940</v>
+        <v>2</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 6 </t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4</v>
+        <v>44444444444</v>
       </c>
       <c r="B5" t="n">
-        <v>44444444444</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
         <v>2</v>
@@ -662,90 +688,108 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F5" t="n">
         <v>4</v>
       </c>
-      <c r="G5" t="n">
-        <v>4</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>4</v>
-      </c>
-      <c r="M5" t="n">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
       </c>
       <c r="N5" t="n">
-        <v>3</v>
+        <v>1488902412421</v>
       </c>
       <c r="O5" t="n">
-        <v>1488902412421</v>
+        <v>133722813124940</v>
       </c>
       <c r="P5" t="n">
-        <v>133722813124940</v>
+        <v>2</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 5 </t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>5</v>
+        <v>55555555555</v>
       </c>
       <c r="B6" t="n">
-        <v>55555555555</v>
+        <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
         <v>3</v>
       </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>1</v>
-      </c>
-      <c r="L6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" t="n">
-        <v>1</v>
-      </c>
       <c r="N6" t="n">
-        <v>3</v>
+        <v>1488902412421</v>
       </c>
       <c r="O6" t="n">
-        <v>1488902412421</v>
+        <v>133722813124940</v>
       </c>
       <c r="P6" t="n">
-        <v>133722813124940</v>
+        <v>2</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4 6 </t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>